<commit_message>
feat(analisis-excel): use docs/AnalisisCredito_Barrera_1116548410_Nano.xlsx as master template
</commit_message>
<xml_diff>
--- a/coodelsur-landing/public/templates/analisis-credito-template.xlsx
+++ b/coodelsur-landing/public/templates/analisis-credito-template.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\REASIGNACION DE CLIENTES\pagares luisa\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\REASIGNACION DE CLIENTES\CLIENTES PARA COMITE\Septiembre\Barrera_1116548410\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1ACE88-A47D-4BFC-ACDA-0FC4CF20632A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Simulador" sheetId="8" r:id="rId1"/>
@@ -42,12 +41,28 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'Evidencia Fotografica'!$2:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Plan de pagos'!$17:$17</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511" refMode="R1C1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>tc={01194A59-06DA-4DC8-B7F5-CDF77A280F33}</author>
     <author>tc={B2750E12-A6E8-447A-BF40-A8C8B00354B6}</author>
@@ -58,7 +73,7 @@
     <author>tc={159544C7-1E6B-496A-AAF1-F11913B8795F}</author>
   </authors>
   <commentList>
-    <comment ref="B16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B16" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -75,7 +90,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B17" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="B17" authorId="1" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +107,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B18" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="B18" authorId="2" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -109,7 +124,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B19" authorId="3" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="B19" authorId="3" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -126,7 +141,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B20" authorId="4" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="B20" authorId="4" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -143,7 +158,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="5" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="B21" authorId="5" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -160,7 +175,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B22" authorId="6" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="B22" authorId="6" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -204,7 +219,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="264">
   <si>
     <t>Intereses</t>
   </si>
@@ -1563,16 +1578,13 @@
     <t>Nanocredito</t>
   </si>
   <si>
-    <t>VARGAS FERNANDEZ JAIME LUIS</t>
-  </si>
-  <si>
-    <t>Mejoras de vivienda</t>
-  </si>
-  <si>
-    <t>Seguridad privada</t>
-  </si>
-  <si>
-    <t>Vigilancia</t>
+    <t>BARRERA RODRIGUEZ  LUZ CARINE</t>
+  </si>
+  <si>
+    <t>Consolidación de Deudas</t>
+  </si>
+  <si>
+    <t>Tienda</t>
   </si>
   <si>
     <r>
@@ -1629,7 +1641,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Email:  jaluva1985@hotmail.com</t>
+      <t>Email:  luzcarine548@gmail.com</t>
     </r>
     <r>
       <rPr>
@@ -1651,7 +1663,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Dirección:  KR 102 25 12 PI 1 102</t>
+      <t>Dirección:  Calle 15 24a 105</t>
     </r>
     <r>
       <rPr>
@@ -1673,7 +1685,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Tel Cel:  3134218571</t>
+      <t>Tel Cel:  3102869287</t>
     </r>
     <r>
       <rPr>
@@ -1695,8 +1707,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Cuenta:3134218571
-Novedad: El cliente dice tener vivienda y vehiculo pero al hacer la respectiva consulta aparece que no cuenta con las dos</t>
+      <t>Cuenta:
+Novedad:</t>
     </r>
     <r>
       <rPr>
@@ -1747,7 +1759,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="11">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
@@ -3899,13 +3911,13 @@
   <cellStyles count="9">
     <cellStyle name="Hipervínculo" xfId="8" builtinId="8"/>
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
-    <cellStyle name="Millares 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Millares 2" xfId="5"/>
     <cellStyle name="Moneda" xfId="6" builtinId="4"/>
     <cellStyle name="Moneda [0]" xfId="7" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal 2" xfId="3"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
-    <cellStyle name="Porcentual 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Porcentual 2" xfId="4"/>
   </cellStyles>
   <dxfs count="15">
     <dxf>
@@ -4046,7 +4058,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Simulador"/>
@@ -4083,9 +4095,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4123,9 +4135,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4160,7 +4172,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4195,7 +4207,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4394,7 +4406,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:O22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4492,7 +4504,7 @@
       </c>
       <c r="F7" s="97" cm="1">
         <f t="array" ref="F7:H7">+'Plan de pagos'!F19:H19</f>
-        <v>116208.58741536846</v>
+        <v>116212.30897513471</v>
       </c>
       <c r="G7" s="100">
         <v>0</v>
@@ -4502,14 +4514,14 @@
       </c>
       <c r="I7" s="82" cm="1">
         <f t="array" ref="I7:J7">+'Plan de pagos'!J19:K19</f>
-        <v>113791.41258463154</v>
+        <v>113787.69102486529</v>
       </c>
       <c r="J7" s="82">
         <v>0</v>
       </c>
       <c r="K7" s="80">
         <f>+'Plan de pagos'!L19</f>
-        <v>4885.6956640380231</v>
+        <v>4900.9002954467996</v>
       </c>
       <c r="L7" s="80">
         <f>+'Plan de pagos'!M19</f>
@@ -4521,11 +4533,11 @@
       </c>
       <c r="N7" s="80">
         <f>+'Plan de pagos'!O19</f>
-        <v>118677.10824866957</v>
+        <v>118688.59132031209</v>
       </c>
       <c r="O7" s="80">
         <f>+'Plan de pagos'!P19</f>
-        <v>144113.62824866956</v>
+        <v>144125.11132031208</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -4547,7 +4559,7 @@
       </c>
       <c r="F8" s="99" cm="1">
         <f t="array" ref="F8:H8">+'Plan de pagos'!F20:H20</f>
-        <v>-2.9103830456733704E-11</v>
+        <v>-1.4551915228366852E-11</v>
       </c>
       <c r="G8" s="83">
         <v>0</v>
@@ -4557,14 +4569,14 @@
       </c>
       <c r="I8" s="82" cm="1">
         <f t="array" ref="I8:J8">+'Plan de pagos'!J20:K20</f>
-        <v>116208.58741536849</v>
+        <v>116212.30897513473</v>
       </c>
       <c r="J8" s="83">
         <v>0</v>
       </c>
       <c r="K8" s="80">
         <f>+'Plan de pagos'!L20</f>
-        <v>2468.5208333010837</v>
+        <v>2476.2823451773584</v>
       </c>
       <c r="L8" s="80">
         <f>+'Plan de pagos'!M20</f>
@@ -4576,11 +4588,11 @@
       </c>
       <c r="N8" s="80">
         <f>+'Plan de pagos'!O20</f>
-        <v>118677.10824866957</v>
+        <v>118688.59132031209</v>
       </c>
       <c r="O8" s="80">
         <f>+'Plan de pagos'!P20</f>
-        <v>144113.62824866956</v>
+        <v>144125.11132031208</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -4593,14 +4605,14 @@
       <c r="H9" s="246"/>
       <c r="I9" s="87" cm="1">
         <f t="array" ref="I9:J9">+'Plan de pagos'!J21:K21</f>
-        <v>230000.00000000003</v>
+        <v>230000</v>
       </c>
       <c r="J9" s="87">
         <v>0</v>
       </c>
       <c r="K9" s="86">
         <f>+'Plan de pagos'!L21</f>
-        <v>7354.2164973391064</v>
+        <v>7377.182640624158</v>
       </c>
       <c r="L9" s="86">
         <f>+'Plan de pagos'!M21</f>
@@ -4612,11 +4624,11 @@
       </c>
       <c r="N9" s="88">
         <f>+'Plan de pagos'!O21</f>
-        <v>237354.21649733913</v>
+        <v>237377.18264062417</v>
       </c>
       <c r="O9" s="88">
         <f>+'Plan de pagos'!P21</f>
-        <v>288227.25649733911</v>
+        <v>288250.22264062415</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -4642,7 +4654,7 @@
       </c>
       <c r="B16" s="92">
         <f>+K9</f>
-        <v>7354.2164973391064</v>
+        <v>7377.182640624158</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -4696,7 +4708,7 @@
       </c>
       <c r="B22" s="91">
         <f>SUM(B15:B21)</f>
-        <v>288227.25649733911</v>
+        <v>288250.22264062415</v>
       </c>
     </row>
   </sheetData>
@@ -4737,7 +4749,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89F8C25-3124-45AB-900F-F844B8996C36}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4844,7 +4856,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:H52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4879,7 +4891,7 @@
       </c>
       <c r="C4" s="3" t="str">
         <f>+'Plan de pagos'!M5</f>
-        <v>VARGAS FERNANDEZ JAIME LUIS</v>
+        <v>BARRERA RODRIGUEZ  LUZ CARINE</v>
       </c>
       <c r="D4" s="2"/>
     </row>
@@ -4889,7 +4901,7 @@
       </c>
       <c r="C5" s="4">
         <f>+'Plan de pagos'!M6</f>
-        <v>1073969021</v>
+        <v>1116548410</v>
       </c>
       <c r="D5" s="2"/>
     </row>
@@ -4899,7 +4911,7 @@
       </c>
       <c r="C6" s="3" t="str">
         <f>+'Plan de pagos'!M7</f>
-        <v>Mejoras de vivienda</v>
+        <v>Consolidación de Deudas</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -4943,7 +4955,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="A1:XEV214"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" zeroHeight="1" x14ac:dyDescent="0.2"/>
@@ -5094,14 +5106,14 @@
         <v>4</v>
       </c>
       <c r="J6" s="16">
-        <v>0.28689999999999999</v>
+        <v>0.28789999999999999</v>
       </c>
       <c r="K6" s="299"/>
       <c r="L6" s="41" t="s">
         <v>24</v>
       </c>
       <c r="M6" s="262">
-        <v>1073969021</v>
+        <v>1116548410</v>
       </c>
       <c r="N6" s="262"/>
       <c r="O6" s="58"/>
@@ -5122,7 +5134,7 @@
       <c r="E7" s="300"/>
       <c r="F7" s="301">
         <f>+J7</f>
-        <v>2.1242155061034884E-2</v>
+        <v>2.130826215411652E-2</v>
       </c>
       <c r="G7" s="302"/>
       <c r="H7" s="303"/>
@@ -5131,7 +5143,7 @@
       </c>
       <c r="J7" s="37">
         <f>((J6+1)^(0.0833333333333333))-1</f>
-        <v>2.1242155061034884E-2</v>
+        <v>2.130826215411652E-2</v>
       </c>
       <c r="K7" s="299"/>
       <c r="L7" s="41" t="s">
@@ -5167,7 +5179,7 @@
       </c>
       <c r="J8" s="38">
         <f>+((1+J7)^3)-1</f>
-        <v>6.5089737717622942E-2</v>
+        <v>6.5296587417168039E-2</v>
       </c>
       <c r="K8" s="299"/>
       <c r="L8" s="41" t="s">
@@ -5204,15 +5216,13 @@
       </c>
       <c r="J9" s="38">
         <f>+J8/(1+J8)</f>
-        <v>6.1111975275532665E-2</v>
+        <v>6.1294280098541258E-2</v>
       </c>
       <c r="K9" s="299"/>
       <c r="L9" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="M9" s="262" t="s">
-        <v>263</v>
-      </c>
+      <c r="M9" s="262"/>
       <c r="N9" s="262"/>
       <c r="O9" s="58"/>
       <c r="P9" s="62">
@@ -5239,7 +5249,7 @@
       </c>
       <c r="J10" s="39">
         <f>+F7*12</f>
-        <v>0.25490586073241861</v>
+        <v>0.25569914584939823</v>
       </c>
       <c r="K10" s="299"/>
       <c r="L10" s="41" t="s">
@@ -5313,7 +5323,7 @@
       </c>
       <c r="O13" s="254"/>
       <c r="P13" s="68">
-        <v>200000</v>
+        <v>500000</v>
       </c>
       <c r="R13" s="15"/>
     </row>
@@ -5467,19 +5477,19 @@
       </c>
       <c r="F19" s="264">
         <f>+(F18-J19)</f>
-        <v>116208.58741536846</v>
+        <v>116212.30897513471</v>
       </c>
       <c r="G19" s="265"/>
       <c r="H19" s="265"/>
       <c r="I19" s="257"/>
       <c r="J19" s="270">
         <f>+($O$19-$L$19)</f>
-        <v>113791.41258463154</v>
+        <v>113787.69102486529</v>
       </c>
       <c r="K19" s="267"/>
       <c r="L19" s="11">
         <f>+(F18*$F$7)</f>
-        <v>4885.6956640380231</v>
+        <v>4900.9002954467996</v>
       </c>
       <c r="M19" s="11">
         <f>IF(J19&gt;0,((+$F$6*1.9)/1000),0)</f>
@@ -5491,11 +5501,11 @@
       </c>
       <c r="O19" s="10">
         <f>+(-PMT($F$7,$F$8,$F$6,0,0))</f>
-        <v>118677.10824866957</v>
+        <v>118688.59132031209</v>
       </c>
       <c r="P19" s="77">
         <f>O19+M19+N19</f>
-        <v>144113.62824866956</v>
+        <v>144125.11132031208</v>
       </c>
       <c r="S19" s="22"/>
     </row>
@@ -5519,19 +5529,19 @@
       </c>
       <c r="F20" s="264">
         <f>IF(F8&lt;=1,0,+F19-J20)</f>
-        <v>-2.9103830456733704E-11</v>
+        <v>-1.4551915228366852E-11</v>
       </c>
       <c r="G20" s="265"/>
       <c r="H20" s="265"/>
       <c r="I20" s="258"/>
       <c r="J20" s="266">
         <f>+IF(F8&lt;=1,0,($O$19-$L$20))</f>
-        <v>116208.58741536849</v>
+        <v>116212.30897513473</v>
       </c>
       <c r="K20" s="267"/>
       <c r="L20" s="11">
         <f>+(F19*$F$7)</f>
-        <v>2468.5208333010837</v>
+        <v>2476.2823451773584</v>
       </c>
       <c r="M20" s="11">
         <f>IF(J20&gt;0,((+$F$6*1.9)/1000),0)</f>
@@ -5543,11 +5553,11 @@
       </c>
       <c r="O20" s="10">
         <f>IF(F8=1,0,(-PMT($F$7,$F$8,$F$6,0,0)))</f>
-        <v>118677.10824866957</v>
+        <v>118688.59132031209</v>
       </c>
       <c r="P20" s="77">
         <f>O20+M20+N20</f>
-        <v>144113.62824866956</v>
+        <v>144125.11132031208</v>
       </c>
       <c r="Q20" s="43"/>
       <c r="S20" s="22"/>
@@ -5564,12 +5574,12 @@
       <c r="I21" s="96"/>
       <c r="J21" s="251">
         <f>+J20+J19</f>
-        <v>230000.00000000003</v>
+        <v>230000</v>
       </c>
       <c r="K21" s="252"/>
       <c r="L21" s="78">
         <f>+L20+L19</f>
-        <v>7354.2164973391064</v>
+        <v>7377.182640624158</v>
       </c>
       <c r="M21" s="78">
         <f>+M20+M19</f>
@@ -5581,11 +5591,11 @@
       </c>
       <c r="O21" s="78">
         <f>+O20+O19</f>
-        <v>237354.21649733913</v>
+        <v>237377.18264062417</v>
       </c>
       <c r="P21" s="90">
         <f>+P20+P19</f>
-        <v>288227.25649733911</v>
+        <v>288250.22264062415</v>
       </c>
     </row>
     <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
@@ -6428,7 +6438,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P7" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P7">
       <formula1>Modalidad</formula1>
     </dataValidation>
   </dataValidations>
@@ -6448,7 +6458,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:H68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -6484,7 +6494,7 @@
       </c>
       <c r="C4" s="1" t="str" cm="1">
         <f t="array" ref="C4:D4">+'Plan de pagos'!M5:N5</f>
-        <v>VARGAS FERNANDEZ JAIME LUIS</v>
+        <v>BARRERA RODRIGUEZ  LUZ CARINE</v>
       </c>
       <c r="D4" s="110">
         <v>0</v>
@@ -6497,7 +6507,7 @@
       </c>
       <c r="C5" s="111" cm="1">
         <f t="array" ref="C5:D5">+'Plan de pagos'!M6:N6</f>
-        <v>1073969021</v>
+        <v>1116548410</v>
       </c>
       <c r="D5" s="110">
         <v>0</v>
@@ -6528,7 +6538,7 @@
         <v>66</v>
       </c>
       <c r="D8" s="117">
-        <v>2600000</v>
+        <v>1700000</v>
       </c>
       <c r="E8" s="118"/>
     </row>
@@ -6537,9 +6547,7 @@
       <c r="C9" s="119" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="117">
-        <v>3011000</v>
-      </c>
+      <c r="D9" s="117"/>
       <c r="E9" s="118"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.2">
@@ -6551,7 +6559,7 @@
       </c>
       <c r="D10" s="120">
         <f>+MIN(D8,D9)</f>
-        <v>2600000</v>
+        <v>1700000</v>
       </c>
       <c r="E10" s="118">
         <f>+D10/D15</f>
@@ -6617,7 +6625,7 @@
       </c>
       <c r="D15" s="125">
         <f>SUM(D10:D14)</f>
-        <v>2600000</v>
+        <v>1700000</v>
       </c>
       <c r="E15" s="126">
         <f>SUM(E10:E14)</f>
@@ -6631,7 +6639,7 @@
       </c>
       <c r="D16" s="125">
         <f>+D15*0.08</f>
-        <v>208000</v>
+        <v>136000</v>
       </c>
       <c r="E16" s="123">
         <f>+D16/D15</f>
@@ -6645,7 +6653,7 @@
       </c>
       <c r="D17" s="128">
         <f>D15-D16</f>
-        <v>2392000</v>
+        <v>1564000</v>
       </c>
       <c r="E17" s="129">
         <f>+D17/D15</f>
@@ -6664,11 +6672,11 @@
       </c>
       <c r="D19" s="130">
         <f>+D17*35%</f>
-        <v>837200</v>
+        <v>547400</v>
       </c>
       <c r="E19" s="118">
         <f>+D19/D26</f>
-        <v>0.5848002235261246</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.2">
@@ -6689,12 +6697,10 @@
       <c r="C21" s="121" t="s">
         <v>80</v>
       </c>
-      <c r="D21" s="133">
-        <v>478400</v>
-      </c>
+      <c r="D21" s="133"/>
       <c r="E21" s="123">
         <f>+D21/D26</f>
-        <v>0.33417155630064266</v>
+        <v>0</v>
       </c>
       <c r="F21" s="132"/>
       <c r="H21" s="125"/>
@@ -6704,12 +6710,10 @@
       <c r="C22" s="121" t="s">
         <v>81</v>
       </c>
-      <c r="D22" s="133">
-        <v>116000</v>
-      </c>
+      <c r="D22" s="133"/>
       <c r="E22" s="123">
         <f>+D22/D26</f>
-        <v>8.1028220173232746E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.2">
@@ -6758,7 +6762,7 @@
       </c>
       <c r="D26" s="128">
         <f>SUM(D19:D25)</f>
-        <v>1431600</v>
+        <v>547400</v>
       </c>
       <c r="E26" s="129">
         <f>SUM(E19:E25)</f>
@@ -6961,7 +6965,7 @@
       <c r="D44" s="137"/>
       <c r="E44" s="154">
         <f>+'Plan de pagos'!P13</f>
-        <v>200000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.2">
@@ -7003,7 +7007,7 @@
       <c r="D47" s="320"/>
       <c r="E47" s="159">
         <f>+'Plan de pagos'!J6</f>
-        <v>0.28689999999999999</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.2">
@@ -7014,7 +7018,7 @@
       <c r="D48" s="305"/>
       <c r="E48" s="161" cm="1">
         <f t="array" ref="E48:G48">+'Plan de pagos'!F7:H7</f>
-        <v>2.1242155061034884E-2</v>
+        <v>2.130826215411652E-2</v>
       </c>
       <c r="F48" s="1">
         <v>0</v>
@@ -7030,7 +7034,7 @@
       </c>
       <c r="E49" s="162">
         <f>+D17-D26</f>
-        <v>960400</v>
+        <v>1016600</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.2">
@@ -7040,7 +7044,7 @@
       </c>
       <c r="E50" s="157">
         <f>+'Plan de pagos'!P19</f>
-        <v>144113.62824866956</v>
+        <v>144125.11132031208</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.2">
@@ -7050,7 +7054,7 @@
       </c>
       <c r="E51" s="157">
         <f>+E49-E50</f>
-        <v>816286.37175133044</v>
+        <v>872474.88867968787</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.2">
@@ -7060,7 +7064,7 @@
       </c>
       <c r="E52" s="157">
         <f>+E51-E65</f>
-        <v>624926.37175133044</v>
+        <v>747354.88867968787</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.2">
@@ -7070,7 +7074,7 @@
       </c>
       <c r="E53" s="163">
         <f>+E50/E49</f>
-        <v>0.15005583949257556</v>
+        <v>0.14177170108234516</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.2">
@@ -7089,7 +7093,7 @@
       </c>
       <c r="E55" s="163">
         <f>(D22+D23+D24)/D17</f>
-        <v>4.8494983277591976E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.2">
@@ -7101,7 +7105,7 @@
       </c>
       <c r="E56" s="163">
         <f>E50/D17</f>
-        <v>6.0248172344761521E-2</v>
+        <v>9.2151605703524347E-2</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.2">
@@ -7111,7 +7115,7 @@
       </c>
       <c r="E57" s="163">
         <f>SUM(D22+D23+D24+E50)/D17</f>
-        <v>0.1087431556223535</v>
+        <v>9.2151605703524347E-2</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.2">
@@ -7150,7 +7154,7 @@
       </c>
       <c r="E61" s="165">
         <f>(E45+D39)/D17</f>
-        <v>8.3612040133779264E-2</v>
+        <v>0.12787723785166241</v>
       </c>
     </row>
     <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -7161,7 +7165,7 @@
       <c r="D62" s="137"/>
       <c r="E62" s="154">
         <f>D17*0.3</f>
-        <v>717600</v>
+        <v>469200</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.2">
@@ -7173,7 +7177,7 @@
       </c>
       <c r="E63" s="157">
         <f>+D17*0.1</f>
-        <v>239200</v>
+        <v>156400</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.2">
@@ -7186,7 +7190,7 @@
       <c r="D64" s="169"/>
       <c r="E64" s="157">
         <f>D17*10</f>
-        <v>23920000</v>
+        <v>15640000</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.2">
@@ -7197,7 +7201,7 @@
       <c r="D65" s="169"/>
       <c r="E65" s="157">
         <f>+D17*0.08</f>
-        <v>191360</v>
+        <v>125120</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.2">
@@ -7207,7 +7211,7 @@
       </c>
       <c r="E66" s="171">
         <f>+E50/30%</f>
-        <v>480378.76082889852</v>
+        <v>480417.03773437359</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.2">
@@ -7218,7 +7222,7 @@
       <c r="D67" s="174"/>
       <c r="E67" s="175">
         <f>(D10+D11)*0.42</f>
-        <v>1092000</v>
+        <v>714000</v>
       </c>
     </row>
     <row r="68" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -7250,7 +7254,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:H32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -7288,14 +7292,14 @@
       </c>
       <c r="C4" s="177" t="str">
         <f>+'Flujo Empleado'!C4</f>
-        <v>VARGAS FERNANDEZ JAIME LUIS</v>
+        <v>BARRERA RODRIGUEZ  LUZ CARINE</v>
       </c>
       <c r="D4" s="178" t="s">
         <v>134</v>
       </c>
       <c r="E4" s="329" t="str">
         <f>+'Plan de pagos'!M8</f>
-        <v>Seguridad privada</v>
+        <v>Tienda</v>
       </c>
       <c r="F4" s="329"/>
       <c r="G4" s="330"/>
@@ -7306,14 +7310,14 @@
       </c>
       <c r="C5" s="180">
         <f>+'Flujo Empleado'!C5</f>
-        <v>1073969021</v>
+        <v>1116548410</v>
       </c>
       <c r="D5" s="181" t="s">
         <v>135</v>
       </c>
-      <c r="E5" s="329" t="str">
+      <c r="E5" s="329">
         <f>+'Plan de pagos'!M9</f>
-        <v>Vigilancia</v>
+        <v>0</v>
       </c>
       <c r="F5" s="329"/>
       <c r="G5" s="330"/>
@@ -7324,7 +7328,7 @@
       </c>
       <c r="C6" s="183" t="str">
         <f>+'Plan de pagos'!M7</f>
-        <v>Mejoras de vivienda</v>
+        <v>Consolidación de Deudas</v>
       </c>
       <c r="D6" s="184" t="s">
         <v>136</v>
@@ -7392,12 +7396,10 @@
       <c r="B11" s="188" t="s">
         <v>140</v>
       </c>
-      <c r="C11" s="189">
-        <v>586</v>
-      </c>
+      <c r="C11" s="189"/>
       <c r="D11" s="324" t="str">
         <f>+IF(C11&lt;500,"Rechazar",(IF(C11&lt;700,"Estudio",IF(C11&gt;=700,"Prestar",0))))</f>
-        <v>Estudio</v>
+        <v>Rechazar</v>
       </c>
       <c r="E11" s="325"/>
       <c r="F11" s="325"/>
@@ -7409,7 +7411,7 @@
       </c>
       <c r="C12" s="190">
         <f>+'Flujo Empleado'!D10</f>
-        <v>2600000</v>
+        <v>1700000</v>
       </c>
       <c r="D12" s="327" t="str">
         <f>+IF(C12&gt;=H12,"Prestar","Rechazado")</f>
@@ -7428,7 +7430,7 @@
       </c>
       <c r="C13" s="192">
         <f>+'Plan de pagos'!P19+'Flujo Empleado'!D26</f>
-        <v>1575713.6282486697</v>
+        <v>691525.11132031213</v>
       </c>
       <c r="D13" s="327" t="str">
         <f>+IF(C13&lt;=C12,"Prestar","Rechazado")</f>
@@ -7445,7 +7447,7 @@
       </c>
       <c r="C14" s="192">
         <f>+C12-C13</f>
-        <v>1024286.3717513303</v>
+        <v>1008474.8886796879</v>
       </c>
       <c r="D14" s="324" t="str">
         <f>+IF(C14&lt;=0,"Rechazado","Prestar")</f>
@@ -7461,11 +7463,11 @@
         <v>155</v>
       </c>
       <c r="C15" s="193" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D15" s="327" t="str">
         <f t="shared" ref="D15" si="0">+IF(C15="SI","Prestar","Rechazado")</f>
-        <v>Prestar</v>
+        <v>Rechazado</v>
       </c>
       <c r="E15" s="327"/>
       <c r="F15" s="327"/>
@@ -7516,10 +7518,10 @@
       </c>
       <c r="C19" s="192">
         <f>+'Plan de pagos'!P13</f>
-        <v>200000</v>
+        <v>500000</v>
       </c>
       <c r="D19" s="342" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E19" s="342"/>
       <c r="F19" s="342"/>
@@ -7698,7 +7700,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15">
       <formula1>$H$17:$H$18</formula1>
     </dataValidation>
   </dataValidations>
@@ -7715,7 +7717,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9004E1B1-790E-4A8A-AB24-17B6BE3686DC}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>ListaDepegable!$C$1:$C$9</xm:f>
           </x14:formula1>
@@ -7728,7 +7730,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7874,15 +7876,15 @@
     <mergeCell ref="B17:C17"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C7" location="Preguntas_Reto!A1" display="Rta. Positiva: De acuerdo (realizar Preguntas reto)" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="E16" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="C7" location="Preguntas_Reto!A1" display="Rta. Positiva: De acuerdo (realizar Preguntas reto)"/>
+    <hyperlink ref="E16" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:Q18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8058,7 +8060,7 @@
     <mergeCell ref="B10:E11"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:E8 B12:E12 B16:E16 G12:J12 G8:J8 G5:J5" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:E8 B12:E12 B16:E16 G12:J12 G8:J8 G5:J5">
       <formula1>$Q$1:$Q$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -8068,7 +8070,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:P49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8429,7 +8431,7 @@
     <mergeCell ref="B21:D21"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D29:E29 D47:E47" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D29:E29 D47:E47">
       <formula1>$P$18:$P$20</formula1>
     </dataValidation>
   </dataValidations>
@@ -8439,7 +8441,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:I58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -8739,7 +8741,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7921A91C-E1DC-4E52-BE31-BA1EC503093F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:D35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8942,8 +8944,8 @@
     <mergeCell ref="C6:C7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C34" r:id="rId1" xr:uid="{E3F1FB2E-9AF1-4558-A5C7-19946178EA9C}"/>
-    <hyperlink ref="C35" r:id="rId2" xr:uid="{E6A26047-6FC6-4608-822F-666126286CE1}"/>
+    <hyperlink ref="C34" r:id="rId1"/>
+    <hyperlink ref="C35" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>